<commit_message>
added testing set up
</commit_message>
<xml_diff>
--- a/uploads/imported_data.xlsx
+++ b/uploads/imported_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliss\OneDrive\Desktop\SusanDB\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF2FF58A-19BC-4C9F-85D0-3B9F9B19BDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB53397E-0C73-436B-9BDF-DB9C61BEFAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4810" yWindow="800" windowWidth="11795" windowHeight="9645" xr2:uid="{97DC95F2-3478-49E5-8D96-4F4A29E57BC1}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{97DC95F2-3478-49E5-8D96-4F4A29E57BC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="E2">
-        <v>3.52</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.75">
@@ -538,7 +538,7 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>3.7</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.75">
@@ -555,7 +555,7 @@
         <v>19</v>
       </c>
       <c r="E5">
-        <v>2.7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new student functionality to import data
</commit_message>
<xml_diff>
--- a/uploads/imported_data.xlsx
+++ b/uploads/imported_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliss\OneDrive\Desktop\SusanDB\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB53397E-0C73-436B-9BDF-DB9C61BEFAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB1A29E-2E83-4945-A580-F6FD8DB9F292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{97DC95F2-3478-49E5-8D96-4F4A29E57BC1}"/>
+    <workbookView xWindow="0" yWindow="1635" windowWidth="19200" windowHeight="9645" xr2:uid="{97DC95F2-3478-49E5-8D96-4F4A29E57BC1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>Non-Binary</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>smith</t>
   </si>
 </sst>
 </file>
@@ -467,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89636726-73D9-4556-9A59-ED29324B9E09}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
@@ -521,7 +527,7 @@
         <v>4</v>
       </c>
       <c r="E3">
-        <v>3.36</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.75">
@@ -538,7 +544,7 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>3.54</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.75">
@@ -556,6 +562,23 @@
       </c>
       <c r="E5">
         <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.75">
+      <c r="A6">
+        <v>124</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reverted new student import data capabilities
</commit_message>
<xml_diff>
--- a/uploads/imported_data.xlsx
+++ b/uploads/imported_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aliss\OneDrive\Desktop\SusanDB\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB1A29E-2E83-4945-A580-F6FD8DB9F292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA1CEB84-EE08-4F71-B6A5-97C8ABDE1A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1635" windowWidth="19200" windowHeight="9645" xr2:uid="{97DC95F2-3478-49E5-8D96-4F4A29E57BC1}"/>
   </bookViews>
@@ -527,7 +527,7 @@
         <v>4</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.75">
@@ -561,12 +561,12 @@
         <v>19</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A6">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>

</xml_diff>